<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-7-8.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-7-8.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-7-8.xlsx
@@ -935,6 +935,9 @@
       <c r="C60" t="str">
         <v>836_胡姬兰紫_undefined_undefined_1bunch</v>
       </c>
+      <c r="F60" t="str">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
@@ -993,7 +996,7 @@
         <v>0.00</v>
       </c>
       <c r="G2" t="str">
-        <v>055555553551010955121510685561587.56108155553040403020101010555555141310101010105520100</v>
+        <v>055555553551010955121510685561587.561081555530404030201010105555551413101010101055201010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>